<commit_message>
feature/fsel-4436: Update Export File Excel Survey
</commit_message>
<xml_diff>
--- a/Services/Fsel.Interaction/Fsel.Interaction.Api/Resources/ExportExcelTemplates/SurveyQuestionReport.xlsx
+++ b/Services/Fsel.Interaction/Fsel.Interaction.Api/Resources/ExportExcelTemplates/SurveyQuestionReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Interaction\Fsel.Interaction.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9DDB5DD-6D3D-4DF6-82DC-1089B7B1F815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4736278B-545D-4A67-BCC2-6771091B508D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{E93CA852-2B0F-43C7-82E9-DD37A9805B82}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -101,12 +101,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -117,12 +111,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFBBC04"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
@@ -130,6 +118,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
@@ -196,41 +190,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -546,117 +534,86 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D17D63B-CBD8-49F6-8499-083FDBB13C42}">
-  <dimension ref="A1:AN4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:40" s="2" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:9" s="9" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
-      <c r="T1" s="7"/>
-      <c r="U1" s="7"/>
-      <c r="V1" s="7"/>
-      <c r="W1" s="7"/>
-      <c r="X1" s="7"/>
-      <c r="Y1" s="7"/>
-      <c r="Z1" s="7"/>
-      <c r="AA1" s="7"/>
-      <c r="AB1" s="7"/>
-      <c r="AC1" s="7"/>
-      <c r="AD1" s="7"/>
-      <c r="AE1" s="7"/>
-      <c r="AF1" s="7"/>
-      <c r="AG1" s="7"/>
-      <c r="AH1" s="7"/>
-      <c r="AI1" s="7"/>
-      <c r="AJ1" s="7"/>
-      <c r="AK1" s="7"/>
-      <c r="AL1" s="7"/>
-      <c r="AM1" s="7"/>
-      <c r="AN1" s="6"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
     </row>
-    <row r="2" spans="1:40" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:40" s="4" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="10" t="s">
+    <row r="3" spans="1:9" s="3" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:40" s="5" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
+    <row r="4" spans="1:9" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
feature/fsel-4436: Update Tool Export Survey
</commit_message>
<xml_diff>
--- a/Services/Fsel.Interaction/Fsel.Interaction.Api/Resources/ExportExcelTemplates/SurveyQuestionReport.xlsx
+++ b/Services/Fsel.Interaction/Fsel.Interaction.Api/Resources/ExportExcelTemplates/SurveyQuestionReport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Interaction\Fsel.Interaction.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4736278B-545D-4A67-BCC2-6771091B508D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814764F9-119F-4005-B385-9485CA8DB289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{E93CA852-2B0F-43C7-82E9-DD37A9805B82}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E93CA852-2B0F-43C7-82E9-DD37A9805B82}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
   <si>
     <t>[{0}] SỐ LIỆU ĐĂNG KÝ &amp; CÂU TRẢ LỜI KHẢO SÁT TRÊN HỆ THỐNG</t>
   </si>
@@ -54,9 +54,6 @@
     <t>tham gia thực tế</t>
   </si>
   <si>
-    <t>đăng ký tài khoản hợp lệ</t>
-  </si>
-  <si>
     <t>Đã hoàn thành PT</t>
   </si>
   <si>
@@ -64,6 +61,15 @@
   </si>
   <si>
     <t>Trả lời Câu hỏi Khảo sát {0}</t>
+  </si>
+  <si>
+    <t>đăng kí tham gia</t>
+  </si>
+  <si>
+    <t>đã xác thực</t>
+  </si>
+  <si>
+    <t>Tỷ lệ</t>
   </si>
 </sst>
 </file>
@@ -202,6 +208,12 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -213,12 +225,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -534,27 +540,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D17D63B-CBD8-49F6-8499-083FDBB13C42}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" s="9" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:11" s="5" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
     </row>
-    <row r="2" spans="1:9" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:11" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -573,60 +581,76 @@
         <v>5</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="J2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" s="3" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="6" t="s">
+    <row r="3" spans="1:11" s="3" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="7"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="J3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="K3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="4" spans="1:9" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
+    <row r="4" spans="1:11" s="4" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="7"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A1:I1"/>
+  <mergeCells count="12">
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="K3:K4"/>
     <mergeCell ref="G3:G4"/>
     <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>